<commit_message>
Osvezi izvestaj (grafici + Excel iz nove baze 7356 zapisa); gitignore scrape logove
</commit_message>
<xml_diff>
--- a/izvestaj/upiti_rezultati.xlsx
+++ b/izvestaj/upiti_rezultati.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="108">
   <si>
     <t>kategorija</t>
   </si>
@@ -31,189 +31,261 @@
     <t>broj_proizvoda</t>
   </si>
   <si>
+    <t>usisivac</t>
+  </si>
+  <si>
     <t>frizider</t>
   </si>
   <si>
+    <t>ves_masina</t>
+  </si>
+  <si>
+    <t>ugradna_rerna</t>
+  </si>
+  <si>
+    <t>pegla</t>
+  </si>
+  <si>
+    <t>sporet</t>
+  </si>
+  <si>
+    <t>masina_za_sudove</t>
+  </si>
+  <si>
+    <t>aspirator</t>
+  </si>
+  <si>
+    <t>mikrotalasna</t>
+  </si>
+  <si>
+    <t>bojler</t>
+  </si>
+  <si>
+    <t>grejno_telo</t>
+  </si>
+  <si>
+    <t>precistac_vazduha</t>
+  </si>
+  <si>
     <t>televizor</t>
   </si>
   <si>
-    <t>ves_masina</t>
-  </si>
-  <si>
-    <t>ugradna_rerna</t>
-  </si>
-  <si>
-    <t>masina_za_sudove</t>
-  </si>
-  <si>
-    <t>mikrotalasna</t>
-  </si>
-  <si>
-    <t>sporet</t>
-  </si>
-  <si>
-    <t>aspirator</t>
-  </si>
-  <si>
-    <t>bojler</t>
+    <t>aparat_za_vodu</t>
   </si>
   <si>
     <t>zamrzivac</t>
   </si>
   <si>
+    <t>aparat_za_kafu</t>
+  </si>
+  <si>
+    <t>ventilator</t>
+  </si>
+  <si>
+    <t>aparat_za_hranu</t>
+  </si>
+  <si>
+    <t>mikser</t>
+  </si>
+  <si>
+    <t>ugradna_ploca</t>
+  </si>
+  <si>
+    <t>toster</t>
+  </si>
+  <si>
+    <t>friteza</t>
+  </si>
+  <si>
+    <t>masina_za_sivenje</t>
+  </si>
+  <si>
+    <t>blender</t>
+  </si>
+  <si>
+    <t>kucni_aparat</t>
+  </si>
+  <si>
+    <t>sokovnik</t>
+  </si>
+  <si>
+    <t>parocistac</t>
+  </si>
+  <si>
+    <t>susilica</t>
+  </si>
+  <si>
+    <t>masina_za_meso</t>
+  </si>
+  <si>
+    <t>seckalica</t>
+  </si>
+  <si>
+    <t>klima_uredjaj</t>
+  </si>
+  <si>
+    <t>reso</t>
+  </si>
+  <si>
+    <t>kuhinjski_robot</t>
+  </si>
+  <si>
+    <t>mini_pekara</t>
+  </si>
+  <si>
     <t>brend</t>
   </si>
   <si>
+    <t>Gorenje</t>
+  </si>
+  <si>
+    <t>Beko</t>
+  </si>
+  <si>
+    <t>Bosch</t>
+  </si>
+  <si>
+    <t>Vox</t>
+  </si>
+  <si>
+    <t>Candy</t>
+  </si>
+  <si>
     <t>VOX</t>
   </si>
   <si>
-    <t>Gorenje</t>
-  </si>
-  <si>
-    <t>Candy</t>
-  </si>
-  <si>
-    <t>Bosch</t>
-  </si>
-  <si>
-    <t>Beko</t>
+    <t>Philips</t>
+  </si>
+  <si>
+    <t>Haier</t>
+  </si>
+  <si>
+    <t>Samsung</t>
+  </si>
+  <si>
+    <t>Electrolux</t>
+  </si>
+  <si>
+    <t>naziv</t>
+  </si>
+  <si>
+    <t>cena</t>
+  </si>
+  <si>
+    <t>dijagonala_inch</t>
+  </si>
+  <si>
+    <t>energetska_klasa</t>
+  </si>
+  <si>
+    <t>Hisense Smart televizor 75E7S PRO</t>
+  </si>
+  <si>
+    <t>Haier Smart televizor H85Q80FUX</t>
+  </si>
+  <si>
+    <t>Samsung Smart televizor QE55S90DAEXXH</t>
+  </si>
+  <si>
+    <t>Hisense Smart televizor 65U8Q</t>
+  </si>
+  <si>
+    <t>LG Smart televizor OLED55B53LA.AEU</t>
+  </si>
+  <si>
+    <t>LG Smart televizor 75NANO81A3A.AEU</t>
+  </si>
+  <si>
+    <t>Haier Smart televizor H75M80FUX</t>
+  </si>
+  <si>
+    <t>Hisense Smart televizor 75U7Q</t>
+  </si>
+  <si>
+    <t>Hisense Smart televizor 75U7SE</t>
+  </si>
+  <si>
+    <t>LG Smart televizor 55" O55B9SLA</t>
+  </si>
+  <si>
+    <t>LG Smart televizor OLED48C31LA.AEU</t>
+  </si>
+  <si>
+    <t>LG Smart televizor OLED48C41LA.AEU</t>
+  </si>
+  <si>
+    <t>LG Smart televizor 65QNED85A3C.AEU</t>
+  </si>
+  <si>
+    <t>Haier Smart televizor H75M90EUX</t>
+  </si>
+  <si>
+    <t>Samsung Smart televizor UE65M80HAUXXH</t>
+  </si>
+  <si>
+    <t>LG Smart televizor 65QNED86A3A.AEU</t>
+  </si>
+  <si>
+    <t>LG Smart televizor OLED48C21LA.AEU</t>
+  </si>
+  <si>
+    <t>Haier Smart televizor H55C95EUX</t>
+  </si>
+  <si>
+    <t>Samsung Smart televizor QE65Q8FAAUXXH</t>
+  </si>
+  <si>
+    <t>Samsung Smart televizor QE55QN70HAUXXH</t>
+  </si>
+  <si>
+    <t>Samsung Smart televizor UE65M70HAUXXH</t>
+  </si>
+  <si>
+    <t>Philips Smart televizor OLED 48OLED769/12</t>
+  </si>
+  <si>
+    <t>Hisense Smart televizor 75E7Q PRO</t>
+  </si>
+  <si>
+    <t>Samsung Smart televizor UE75U8072FUXXH</t>
+  </si>
+  <si>
+    <t>LG Smart televizor 65QNED80A3A.AEU</t>
+  </si>
+  <si>
+    <t>Hisense Smart televizor 55U8Q</t>
+  </si>
+  <si>
+    <t>Hisense Smart televizor 65E7S PRO</t>
+  </si>
+  <si>
+    <t>LG Smart televizor 55QNED85A3C.AEU</t>
+  </si>
+  <si>
+    <t>Hisense Smart televizor 75Q7S</t>
+  </si>
+  <si>
+    <t>Hisense Smart televizor 75A7Q</t>
+  </si>
+  <si>
+    <t>Hisense</t>
   </si>
   <si>
     <t>LG</t>
   </si>
   <si>
-    <t>Haier</t>
-  </si>
-  <si>
-    <t>Samsung</t>
-  </si>
-  <si>
-    <t>Hisense</t>
-  </si>
-  <si>
-    <t>Whirlpool</t>
-  </si>
-  <si>
-    <t>naziv</t>
-  </si>
-  <si>
-    <t>cena</t>
-  </si>
-  <si>
-    <t>dijagonala_inch</t>
-  </si>
-  <si>
-    <t>energetska_klasa</t>
-  </si>
-  <si>
-    <t>Hisense Smart televizor 116UXQ</t>
-  </si>
-  <si>
-    <t>SAMSUNG Smart TV QE98QN90AATXXH</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor QE65QN900BTXXH</t>
-  </si>
-  <si>
-    <t>LG Smart televizor OLED77G51LW.AEU</t>
-  </si>
-  <si>
-    <t>LG Smart televizor OLED65M59LA.AEU</t>
-  </si>
-  <si>
-    <t>LG Smart televizor OLED77C51LA.AEU</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor QE65S90HAEXXH</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor QE75LS03FWUXXH</t>
-  </si>
-  <si>
-    <t>LG Smart televizor  OLED65G53LS.AEU</t>
-  </si>
-  <si>
-    <t>Hisense Smart televizor 100E7S PRO</t>
-  </si>
-  <si>
-    <t>LG Smart televizor OLED65G51LW.AEU</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor QE65QN700BTXXH</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor QE65QN800BTXXH</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor MRE65R85HAUXXH</t>
-  </si>
-  <si>
-    <t>LG Smart televizor OLED65G23LA</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor QE55S90HAEXXH</t>
-  </si>
-  <si>
-    <t>Haier Smart televizor H98S900UX</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor MRE55R85HAUXXH</t>
-  </si>
-  <si>
-    <t>LG Smart televizor OLED55G53LS.AEU</t>
-  </si>
-  <si>
-    <t>LG Smart televizor OLED55G51LW.AEU</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor QE55S95FATXXH</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor QE65Q85RATXXH</t>
-  </si>
-  <si>
-    <t>LG Smart televizor OLED65C51LA.AEU</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor QE55S95CATXXH</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor QE55Q85RATXXH</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor QE55QN95DATXXH</t>
-  </si>
-  <si>
-    <t>LG Smart televizor OLED55G42LW</t>
-  </si>
-  <si>
-    <t>LG Smart televizor OLED55G23LA.AEU</t>
-  </si>
-  <si>
-    <t>LG Smart televizor 86NANO81A3A.AEU</t>
-  </si>
-  <si>
-    <t>Samsung Smart televizor UE75M80HAUXXH</t>
-  </si>
-  <si>
-    <t>SAMSUNG</t>
+    <t>F</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>E</t>
   </si>
   <si>
     <t>D</t>
   </si>
   <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>G</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>B (po prethodnoj klasifikaciji)</t>
-  </si>
-  <si>
     <t>prosecna_cena</t>
   </si>
   <si>
@@ -229,13 +301,31 @@
     <t>ukupno</t>
   </si>
   <si>
-    <t>klasa_A_ili_bolja</t>
-  </si>
-  <si>
-    <t>procenat_klasa_A</t>
-  </si>
-  <si>
-    <t>Indesit</t>
+    <t>klasa_a_ili_bolja</t>
+  </si>
+  <si>
+    <t>procenat_klasa_a</t>
+  </si>
+  <si>
+    <t>Alfa Plam</t>
+  </si>
+  <si>
+    <t>Milan Blagojevic</t>
+  </si>
+  <si>
+    <t>Roborock</t>
+  </si>
+  <si>
+    <t>Aeg</t>
+  </si>
+  <si>
+    <t>Dyson</t>
+  </si>
+  <si>
+    <t>TCL</t>
+  </si>
+  <si>
+    <t>Dreame</t>
   </si>
   <si>
     <t>na_lageru</t>
@@ -588,7 +678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -604,7 +694,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>231</v>
+        <v>975</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -612,7 +702,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>211</v>
+        <v>814</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -620,7 +710,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>204</v>
+        <v>708</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -628,7 +718,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>141</v>
+        <v>685</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -636,7 +726,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>110</v>
+        <v>515</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -644,7 +734,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>77</v>
+        <v>494</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -652,7 +742,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>67</v>
+        <v>468</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -660,7 +750,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>57</v>
+        <v>338</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -668,7 +758,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>34</v>
+        <v>260</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -676,7 +766,199 @@
         <v>11</v>
       </c>
       <c r="B11">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" t="s">
         <v>29</v>
+      </c>
+      <c r="B29">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -691,46 +973,46 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>74</v>
+        <v>104</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="B2">
-        <v>74</v>
+        <v>229</v>
       </c>
       <c r="C2">
-        <v>28908</v>
+        <v>37207</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>106</v>
       </c>
       <c r="B3">
-        <v>149</v>
+        <v>404</v>
       </c>
       <c r="C3">
-        <v>78968</v>
+        <v>60487</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>107</v>
       </c>
       <c r="B4">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="C4">
-        <v>172315</v>
+        <v>84230</v>
       </c>
     </row>
   </sheetData>
@@ -745,7 +1027,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -753,82 +1035,82 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>169</v>
+        <v>833</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>139</v>
+        <v>536</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>128</v>
+        <v>527</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="B5">
-        <v>104</v>
+        <v>439</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="B6">
-        <v>96</v>
+        <v>403</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="B7">
-        <v>86</v>
+        <v>361</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="B8">
-        <v>83</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="B9">
-        <v>73</v>
+        <v>192</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="B10">
-        <v>56</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="B11">
-        <v>37</v>
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -848,7 +1130,7 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2">
-        <v>181</v>
+        <v>1508</v>
       </c>
     </row>
   </sheetData>
@@ -868,7 +1150,7 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2">
-        <v>708</v>
+        <v>5758</v>
       </c>
     </row>
   </sheetData>
@@ -883,529 +1165,517 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="B1" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="D1" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="E1" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="C2">
-        <v>2499999</v>
-      </c>
-      <c r="D2">
-        <v>116</v>
-      </c>
-      <c r="E2" t="s">
-        <v>58</v>
+        <v>119999</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="C3">
-        <v>1249977</v>
+        <v>119999</v>
       </c>
       <c r="D3">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C4">
-        <v>479999</v>
+        <v>119844</v>
       </c>
       <c r="D4">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>81</v>
       </c>
       <c r="C5">
-        <v>379999</v>
+        <v>114999</v>
       </c>
       <c r="D5">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>82</v>
       </c>
       <c r="C6">
-        <v>369999</v>
+        <v>114999</v>
       </c>
       <c r="D6">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="E6" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>82</v>
       </c>
       <c r="C7">
-        <v>279999</v>
+        <v>109999</v>
       </c>
       <c r="D7">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E7" t="s">
-        <v>61</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="C8">
-        <v>269999</v>
+        <v>109999</v>
       </c>
       <c r="D8">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>81</v>
       </c>
       <c r="C9">
-        <v>259999</v>
+        <v>109999</v>
       </c>
       <c r="D9">
         <v>75</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>81</v>
       </c>
       <c r="C10">
-        <v>249999</v>
+        <v>109999</v>
       </c>
       <c r="D10">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>82</v>
       </c>
       <c r="C11">
-        <v>249999</v>
-      </c>
-      <c r="D11">
-        <v>100</v>
-      </c>
-      <c r="E11" t="s">
-        <v>59</v>
+        <v>109977</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>82</v>
       </c>
       <c r="C12">
-        <v>249999</v>
+        <v>109977</v>
       </c>
       <c r="D12">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>82</v>
       </c>
       <c r="C13">
-        <v>249977</v>
+        <v>109977</v>
       </c>
       <c r="D13">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="E13" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>39</v>
+        <v>63</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>82</v>
       </c>
       <c r="C14">
-        <v>249977</v>
+        <v>99999</v>
       </c>
       <c r="D14">
         <v>65</v>
       </c>
       <c r="E14" t="s">
-        <v>60</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="B15" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="C15">
-        <v>239999</v>
+        <v>99999</v>
       </c>
       <c r="D15">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="E15" t="s">
-        <v>61</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="C16">
-        <v>234977</v>
+        <v>99999</v>
       </c>
       <c r="D16">
         <v>65</v>
       </c>
       <c r="E16" t="s">
-        <v>61</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>82</v>
       </c>
       <c r="C17">
-        <v>219999</v>
+        <v>99999</v>
       </c>
       <c r="D17">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="B18" t="s">
-        <v>19</v>
+        <v>82</v>
       </c>
       <c r="C18">
-        <v>209999</v>
+        <v>99977</v>
       </c>
       <c r="D18">
-        <v>98</v>
+        <v>48</v>
       </c>
       <c r="E18" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" t="s">
         <v>44</v>
       </c>
-      <c r="B19" t="s">
-        <v>20</v>
-      </c>
       <c r="C19">
-        <v>204999</v>
+        <v>89999</v>
       </c>
       <c r="D19">
         <v>55</v>
       </c>
       <c r="E19" t="s">
-        <v>61</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" t="s">
         <v>45</v>
       </c>
-      <c r="B20" t="s">
-        <v>18</v>
-      </c>
       <c r="C20">
-        <v>199999</v>
+        <v>89999</v>
       </c>
       <c r="D20">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="E20" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="B21" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="C21">
-        <v>199999</v>
+        <v>89999</v>
       </c>
       <c r="D21">
         <v>55</v>
       </c>
       <c r="E21" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="B22" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C22">
-        <v>199999</v>
+        <v>89999</v>
       </c>
       <c r="D22">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="E22" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C23">
+        <v>89977</v>
+      </c>
+      <c r="D23">
         <v>48</v>
       </c>
-      <c r="B23" t="s">
-        <v>20</v>
-      </c>
-      <c r="C23">
-        <v>199977</v>
-      </c>
-      <c r="D23">
-        <v>65</v>
-      </c>
       <c r="E23" t="s">
-        <v>62</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="B24" t="s">
-        <v>18</v>
+        <v>81</v>
       </c>
       <c r="C24">
-        <v>189999</v>
+        <v>87999</v>
       </c>
       <c r="D24">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="E24" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" t="s">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="B25" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="C25">
-        <v>189999</v>
+        <v>84999</v>
       </c>
       <c r="D25">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="E25" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="B26" t="s">
-        <v>20</v>
+        <v>82</v>
       </c>
       <c r="C26">
-        <v>179977</v>
+        <v>84999</v>
       </c>
       <c r="D26">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="E26" t="s">
-        <v>62</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="B27" t="s">
-        <v>20</v>
+        <v>81</v>
       </c>
       <c r="C27">
-        <v>179977</v>
+        <v>82844</v>
       </c>
       <c r="D27">
         <v>55</v>
       </c>
       <c r="E27" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="B28" t="s">
-        <v>18</v>
+        <v>81</v>
       </c>
       <c r="C28">
-        <v>179977</v>
+        <v>79999</v>
       </c>
       <c r="D28">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="E28" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29" t="s">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="B29" t="s">
-        <v>18</v>
+        <v>82</v>
       </c>
       <c r="C29">
-        <v>169977</v>
+        <v>79999</v>
       </c>
       <c r="D29">
         <v>55</v>
       </c>
       <c r="E29" t="s">
-        <v>60</v>
+        <v>85</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
       <c r="B30" t="s">
-        <v>18</v>
+        <v>81</v>
       </c>
       <c r="C30">
-        <v>159999</v>
+        <v>79999</v>
       </c>
       <c r="D30">
-        <v>86</v>
+        <v>75</v>
       </c>
       <c r="E30" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="B31" t="s">
-        <v>20</v>
+        <v>81</v>
       </c>
       <c r="C31">
-        <v>159999</v>
+        <v>79999</v>
       </c>
       <c r="D31">
         <v>75</v>
       </c>
       <c r="E31" t="s">
-        <v>58</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1415,7 +1685,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1426,56 +1696,56 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="D1" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="E1" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="F1" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="B2">
-        <v>211</v>
+        <v>171</v>
       </c>
       <c r="C2">
-        <v>102480.53</v>
+        <v>55705.95</v>
       </c>
       <c r="D2">
         <v>10999</v>
       </c>
       <c r="E2">
-        <v>2499999</v>
+        <v>119999</v>
       </c>
       <c r="F2">
-        <v>197185.4</v>
+        <v>26593.52</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="B3">
-        <v>231</v>
+        <v>27</v>
       </c>
       <c r="C3">
-        <v>65107.13</v>
+        <v>53396.15</v>
       </c>
       <c r="D3">
-        <v>99</v>
+        <v>27999</v>
       </c>
       <c r="E3">
-        <v>333999</v>
+        <v>89999</v>
       </c>
       <c r="F3">
-        <v>56996.42</v>
+        <v>20281.67</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1483,79 +1753,79 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>204</v>
+        <v>708</v>
       </c>
       <c r="C4">
-        <v>63137.45</v>
+        <v>53193.78</v>
       </c>
       <c r="D4">
-        <v>26999</v>
+        <v>1299</v>
       </c>
       <c r="E4">
-        <v>209999</v>
+        <v>119999</v>
       </c>
       <c r="F4">
-        <v>33544.06</v>
+        <v>22273.11</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B5">
-        <v>141</v>
+        <v>814</v>
       </c>
       <c r="C5">
-        <v>51400.26</v>
+        <v>49516.23</v>
       </c>
       <c r="D5">
-        <v>13999</v>
+        <v>1099</v>
       </c>
       <c r="E5">
-        <v>261499</v>
+        <v>120990</v>
       </c>
       <c r="F5">
-        <v>42652.77</v>
+        <v>27892.65</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B6">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="C6">
-        <v>49076.24</v>
+        <v>49051.76</v>
       </c>
       <c r="D6">
-        <v>19999</v>
+        <v>28341</v>
       </c>
       <c r="E6">
-        <v>153999</v>
+        <v>87866</v>
       </c>
       <c r="F6">
-        <v>32565.92</v>
+        <v>13976.62</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7">
-        <v>110</v>
+        <v>494</v>
       </c>
       <c r="C7">
-        <v>47559.01</v>
+        <v>48035.53</v>
       </c>
       <c r="D7">
-        <v>27144</v>
+        <v>1099</v>
       </c>
       <c r="E7">
-        <v>99899</v>
+        <v>115499</v>
       </c>
       <c r="F7">
-        <v>16556.27</v>
+        <v>27676.69</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1563,79 +1833,559 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>67</v>
+        <v>468</v>
       </c>
       <c r="C8">
-        <v>28858.1</v>
+        <v>46427.7</v>
       </c>
       <c r="D8">
-        <v>1299</v>
+        <v>3299</v>
       </c>
       <c r="E8">
-        <v>88999</v>
+        <v>120999</v>
       </c>
       <c r="F8">
-        <v>19202.23</v>
+        <v>17773.26</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B9">
-        <v>57</v>
+        <v>125</v>
       </c>
       <c r="C9">
-        <v>22829.16</v>
+        <v>39989.13</v>
       </c>
       <c r="D9">
-        <v>6244</v>
+        <v>15899</v>
       </c>
       <c r="E9">
-        <v>111999</v>
+        <v>119499</v>
       </c>
       <c r="F9">
-        <v>24914.85</v>
+        <v>19592.61</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B10">
-        <v>77</v>
+        <v>685</v>
       </c>
       <c r="C10">
-        <v>22238.78</v>
+        <v>39428.94</v>
       </c>
       <c r="D10">
-        <v>6599</v>
+        <v>3199</v>
       </c>
       <c r="E10">
-        <v>184999</v>
+        <v>118999</v>
       </c>
       <c r="F10">
-        <v>30235.49</v>
+        <v>18658.84</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11">
+        <v>70</v>
+      </c>
+      <c r="C11">
+        <v>39423.29</v>
+      </c>
+      <c r="D11">
+        <v>14999</v>
+      </c>
+      <c r="E11">
+        <v>84999</v>
+      </c>
+      <c r="F11">
+        <v>16067.77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12">
+        <v>19</v>
+      </c>
+      <c r="C12">
+        <v>32828.84</v>
+      </c>
+      <c r="D12">
+        <v>8999</v>
+      </c>
+      <c r="E12">
+        <v>105999</v>
+      </c>
+      <c r="F12">
+        <v>26740.31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13">
+        <v>86</v>
+      </c>
+      <c r="C13">
+        <v>31684.99</v>
+      </c>
+      <c r="D13">
+        <v>9891</v>
+      </c>
+      <c r="E13">
+        <v>100990</v>
+      </c>
+      <c r="F13">
+        <v>16735.07</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14">
+        <v>179</v>
+      </c>
+      <c r="C14">
+        <v>29242.17</v>
+      </c>
+      <c r="D14">
+        <v>1096</v>
+      </c>
+      <c r="E14">
+        <v>109999</v>
+      </c>
+      <c r="F14">
+        <v>30341.51</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15">
+        <v>975</v>
+      </c>
+      <c r="C15">
+        <v>25522.68</v>
+      </c>
+      <c r="D15">
+        <v>1077</v>
+      </c>
+      <c r="E15">
+        <v>119999</v>
+      </c>
+      <c r="F15">
+        <v>26605.62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16">
+        <v>338</v>
+      </c>
+      <c r="C16">
+        <v>23876.65</v>
+      </c>
+      <c r="D16">
+        <v>1199</v>
+      </c>
+      <c r="E16">
+        <v>119069</v>
+      </c>
+      <c r="F16">
+        <v>24697.08</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17">
+        <v>177</v>
+      </c>
+      <c r="C17">
+        <v>22005.44</v>
+      </c>
+      <c r="D17">
+        <v>1299</v>
+      </c>
+      <c r="E17">
+        <v>109999</v>
+      </c>
+      <c r="F17">
+        <v>23215.94</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18">
+        <v>193</v>
+      </c>
+      <c r="C18">
+        <v>21086.36</v>
+      </c>
+      <c r="D18">
+        <v>5999</v>
+      </c>
+      <c r="E18">
+        <v>120999</v>
+      </c>
+      <c r="F18">
+        <v>13445.81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19">
+        <v>8</v>
+      </c>
+      <c r="C19">
+        <v>20874</v>
+      </c>
+      <c r="D19">
+        <v>10099</v>
+      </c>
+      <c r="E19">
+        <v>39199</v>
+      </c>
+      <c r="F19">
+        <v>10700.43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20">
+        <v>122</v>
+      </c>
+      <c r="C20">
+        <v>20491.64</v>
+      </c>
+      <c r="D20">
+        <v>1099</v>
+      </c>
+      <c r="E20">
+        <v>94199</v>
+      </c>
+      <c r="F20">
+        <v>24048.79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" t="s">
         <v>10</v>
       </c>
-      <c r="B11">
+      <c r="B21">
+        <v>260</v>
+      </c>
+      <c r="C21">
+        <v>20171.65</v>
+      </c>
+      <c r="D21">
+        <v>5999</v>
+      </c>
+      <c r="E21">
+        <v>109999</v>
+      </c>
+      <c r="F21">
+        <v>17603.88</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22">
+        <v>42</v>
+      </c>
+      <c r="C22">
+        <v>15976.38</v>
+      </c>
+      <c r="D22">
+        <v>1199</v>
+      </c>
+      <c r="E22">
+        <v>63249</v>
+      </c>
+      <c r="F22">
+        <v>13605.84</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23">
+        <v>71</v>
+      </c>
+      <c r="C23">
+        <v>15952.32</v>
+      </c>
+      <c r="D23">
+        <v>1877</v>
+      </c>
+      <c r="E23">
+        <v>49277</v>
+      </c>
+      <c r="F23">
+        <v>9270.110000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24">
+        <v>44</v>
+      </c>
+      <c r="C24">
+        <v>15634.55</v>
+      </c>
+      <c r="D24">
+        <v>1599</v>
+      </c>
+      <c r="E24">
+        <v>74999</v>
+      </c>
+      <c r="F24">
+        <v>18787.51</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25">
         <v>34</v>
       </c>
-      <c r="C11">
-        <v>16479.88</v>
-      </c>
-      <c r="D11">
-        <v>5999</v>
-      </c>
-      <c r="E11">
-        <v>37999</v>
-      </c>
-      <c r="F11">
-        <v>7444.65</v>
+      <c r="C25">
+        <v>13236.79</v>
+      </c>
+      <c r="D25">
+        <v>4499</v>
+      </c>
+      <c r="E25">
+        <v>36499</v>
+      </c>
+      <c r="F25">
+        <v>6147.83</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26">
+        <v>44</v>
+      </c>
+      <c r="C26">
+        <v>11662.64</v>
+      </c>
+      <c r="D26">
+        <v>1199</v>
+      </c>
+      <c r="E26">
+        <v>110999</v>
+      </c>
+      <c r="F26">
+        <v>16971.67</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27">
+        <v>515</v>
+      </c>
+      <c r="C27">
+        <v>11448.27</v>
+      </c>
+      <c r="D27">
+        <v>1039</v>
+      </c>
+      <c r="E27">
+        <v>99199</v>
+      </c>
+      <c r="F27">
+        <v>13512.83</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>18</v>
+      </c>
+      <c r="B28">
+        <v>120</v>
+      </c>
+      <c r="C28">
+        <v>11283.92</v>
+      </c>
+      <c r="D28">
+        <v>2499</v>
+      </c>
+      <c r="E28">
+        <v>65499</v>
+      </c>
+      <c r="F28">
+        <v>10078.66</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>25</v>
+      </c>
+      <c r="B29">
+        <v>57</v>
+      </c>
+      <c r="C29">
+        <v>9812.860000000001</v>
+      </c>
+      <c r="D29">
+        <v>1999</v>
+      </c>
+      <c r="E29">
+        <v>73999</v>
+      </c>
+      <c r="F29">
+        <v>10520.32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
+        <v>33</v>
+      </c>
+      <c r="B30">
+        <v>22</v>
+      </c>
+      <c r="C30">
+        <v>6757.09</v>
+      </c>
+      <c r="D30">
+        <v>2299</v>
+      </c>
+      <c r="E30">
+        <v>19199</v>
+      </c>
+      <c r="F30">
+        <v>4634.76</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" t="s">
+        <v>19</v>
+      </c>
+      <c r="B31">
+        <v>112</v>
+      </c>
+      <c r="C31">
+        <v>6690.15</v>
+      </c>
+      <c r="D31">
+        <v>1099</v>
+      </c>
+      <c r="E31">
+        <v>53199</v>
+      </c>
+      <c r="F31">
+        <v>8046.16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32">
+        <v>100</v>
+      </c>
+      <c r="C32">
+        <v>5162.49</v>
+      </c>
+      <c r="D32">
+        <v>1199</v>
+      </c>
+      <c r="E32">
+        <v>23899</v>
+      </c>
+      <c r="F32">
+        <v>3436.17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" t="s">
+        <v>22</v>
+      </c>
+      <c r="B33">
+        <v>74</v>
+      </c>
+      <c r="C33">
+        <v>4093.16</v>
+      </c>
+      <c r="D33">
+        <v>1599</v>
+      </c>
+      <c r="E33">
+        <v>16999</v>
+      </c>
+      <c r="F33">
+        <v>2378.79</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" t="s">
+        <v>15</v>
+      </c>
+      <c r="B34">
+        <v>129</v>
+      </c>
+      <c r="C34">
+        <v>4014.19</v>
+      </c>
+      <c r="D34">
+        <v>1177</v>
+      </c>
+      <c r="E34">
+        <v>69999</v>
+      </c>
+      <c r="F34">
+        <v>6413.37</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35">
+        <v>32</v>
+      </c>
+      <c r="C35">
+        <v>3850.75</v>
+      </c>
+      <c r="D35">
+        <v>1699</v>
+      </c>
+      <c r="E35">
+        <v>10799</v>
+      </c>
+      <c r="F35">
+        <v>1939.63</v>
       </c>
     </row>
   </sheetData>
@@ -1645,7 +2395,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1653,24 +2403,24 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="C1" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="D1" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>283</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>283</v>
       </c>
       <c r="D2">
         <v>100</v>
@@ -1678,13 +2428,13 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C3">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D3">
         <v>100</v>
@@ -1692,99 +2442,169 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D4">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="B5">
-        <v>188</v>
+        <v>305</v>
       </c>
       <c r="C5">
-        <v>90</v>
+        <v>301</v>
       </c>
       <c r="D5">
-        <v>47.9</v>
+        <v>98.7</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B6">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D6">
-        <v>13.3</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B7">
-        <v>110</v>
+        <v>23</v>
       </c>
       <c r="C7">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="D7">
-        <v>4.5</v>
+        <v>69.59999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B8">
-        <v>204</v>
+        <v>666</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>364</v>
       </c>
       <c r="D8">
-        <v>0.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B9">
-        <v>209</v>
+        <v>164</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>20.7</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B10">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="C10">
+        <v>7</v>
+      </c>
+      <c r="D10">
+        <v>17.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>204</v>
+      </c>
+      <c r="C11">
+        <v>33</v>
+      </c>
+      <c r="D11">
+        <v>16.2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12">
+        <v>459</v>
+      </c>
+      <c r="C12">
+        <v>15</v>
+      </c>
+      <c r="D12">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13">
+        <v>751</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14">
+        <v>125</v>
+      </c>
+      <c r="C14">
         <v>0</v>
       </c>
-      <c r="D10">
+      <c r="D14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>165</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
         <v>0</v>
       </c>
     </row>
@@ -1800,189 +2620,189 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="D1" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="E1" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>94</v>
       </c>
       <c r="B2">
-        <v>56</v>
+        <v>102</v>
       </c>
       <c r="C2">
-        <v>120926</v>
+        <v>75353</v>
       </c>
       <c r="D2">
-        <v>9999</v>
+        <v>21899</v>
       </c>
       <c r="E2">
-        <v>2499999</v>
+        <v>105499</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>95</v>
       </c>
       <c r="B3">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="C3">
-        <v>109219</v>
+        <v>72947</v>
       </c>
       <c r="D3">
-        <v>13844</v>
+        <v>21999</v>
       </c>
       <c r="E3">
-        <v>379999</v>
+        <v>115499</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>96</v>
       </c>
       <c r="B4">
-        <v>73</v>
+        <v>22</v>
       </c>
       <c r="C4">
-        <v>99244</v>
+        <v>69454</v>
       </c>
       <c r="D4">
-        <v>8399</v>
+        <v>32999</v>
       </c>
       <c r="E4">
-        <v>479999</v>
+        <v>119999</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>97</v>
       </c>
       <c r="B5">
-        <v>104</v>
+        <v>29</v>
       </c>
       <c r="C5">
-        <v>96692</v>
+        <v>68982</v>
       </c>
       <c r="D5">
-        <v>16499</v>
+        <v>17999</v>
       </c>
       <c r="E5">
-        <v>333999</v>
+        <v>115999</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="B6">
-        <v>83</v>
+        <v>192</v>
       </c>
       <c r="C6">
-        <v>85836</v>
+        <v>68022</v>
       </c>
       <c r="D6">
-        <v>23999</v>
+        <v>5999</v>
       </c>
       <c r="E6">
-        <v>244799</v>
+        <v>119999</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>82</v>
       </c>
       <c r="B7">
-        <v>37</v>
+        <v>112</v>
       </c>
       <c r="C7">
-        <v>56632</v>
+        <v>65269</v>
       </c>
       <c r="D7">
-        <v>13999</v>
+        <v>11499</v>
       </c>
       <c r="E7">
-        <v>96899</v>
+        <v>119999</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="B8">
-        <v>26</v>
+        <v>104</v>
       </c>
       <c r="C8">
-        <v>41648</v>
+        <v>59775</v>
       </c>
       <c r="D8">
-        <v>16799</v>
+        <v>8999</v>
       </c>
       <c r="E8">
-        <v>84344</v>
+        <v>119999</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>98</v>
       </c>
       <c r="B9">
-        <v>96</v>
+        <v>47</v>
       </c>
       <c r="C9">
-        <v>41077</v>
+        <v>55044</v>
       </c>
       <c r="D9">
-        <v>9199</v>
+        <v>7599</v>
       </c>
       <c r="E9">
-        <v>103999</v>
+        <v>119999</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>99</v>
       </c>
       <c r="B10">
-        <v>139</v>
+        <v>29</v>
       </c>
       <c r="C10">
-        <v>39031</v>
+        <v>53045</v>
       </c>
       <c r="D10">
-        <v>7299</v>
+        <v>3999</v>
       </c>
       <c r="E10">
-        <v>145799</v>
+        <v>109999</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="B11">
-        <v>128</v>
+        <v>35</v>
       </c>
       <c r="C11">
-        <v>36624</v>
+        <v>51302</v>
       </c>
       <c r="D11">
-        <v>7599</v>
+        <v>15999</v>
       </c>
       <c r="E11">
-        <v>102799</v>
+        <v>88299</v>
       </c>
     </row>
   </sheetData>
@@ -1992,7 +2812,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2000,27 +2820,27 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="C1" t="s">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="D1" t="s">
-        <v>72</v>
+        <v>102</v>
       </c>
       <c r="E1" t="s">
-        <v>73</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B2">
-        <v>57</v>
+        <v>112</v>
       </c>
       <c r="C2">
-        <v>57</v>
+        <v>112</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -2031,13 +2851,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="B3">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="C3">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -2048,13 +2868,13 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="B4">
-        <v>110</v>
+        <v>74</v>
       </c>
       <c r="C4">
-        <v>110</v>
+        <v>74</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -2065,13 +2885,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B5">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="C5">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -2082,13 +2902,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="B6">
-        <v>67</v>
+        <v>34</v>
       </c>
       <c r="C6">
-        <v>67</v>
+        <v>34</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -2099,13 +2919,13 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B7">
-        <v>211</v>
+        <v>338</v>
       </c>
       <c r="C7">
-        <v>211</v>
+        <v>338</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -2116,13 +2936,13 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B8">
-        <v>29</v>
+        <v>122</v>
       </c>
       <c r="C8">
-        <v>29</v>
+        <v>122</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -2133,53 +2953,461 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="B9">
-        <v>203</v>
+        <v>129</v>
       </c>
       <c r="C9">
-        <v>202</v>
+        <v>129</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>99.5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="B10">
-        <v>230</v>
+        <v>27</v>
       </c>
       <c r="C10">
-        <v>227</v>
+        <v>27</v>
       </c>
       <c r="D10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>98.7</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11">
+        <v>41</v>
+      </c>
+      <c r="C11">
+        <v>41</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12">
+        <v>100</v>
+      </c>
+      <c r="C12">
+        <v>100</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13">
+        <v>8</v>
+      </c>
+      <c r="C13">
+        <v>8</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14">
+        <v>32</v>
+      </c>
+      <c r="C14">
+        <v>32</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>171</v>
+      </c>
+      <c r="C15">
+        <v>171</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16">
+        <v>193</v>
+      </c>
+      <c r="C16">
+        <v>193</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17">
+        <v>71</v>
+      </c>
+      <c r="C17">
+        <v>71</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18">
+        <v>86</v>
+      </c>
+      <c r="C18">
+        <v>86</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19">
+        <v>42</v>
+      </c>
+      <c r="C19">
+        <v>42</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20">
+        <v>22</v>
+      </c>
+      <c r="C20">
+        <v>22</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21">
+        <v>468</v>
+      </c>
+      <c r="C21">
+        <v>467</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <v>99.8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22">
+        <v>494</v>
+      </c>
+      <c r="C22">
+        <v>493</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22">
+        <v>99.8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>10</v>
+      </c>
+      <c r="B23">
+        <v>260</v>
+      </c>
+      <c r="C23">
+        <v>259</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>99.59999999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" t="s">
+        <v>4</v>
+      </c>
+      <c r="B24">
+        <v>708</v>
+      </c>
+      <c r="C24">
+        <v>703</v>
+      </c>
+      <c r="D24">
         <v>5</v>
       </c>
-      <c r="B11">
-        <v>141</v>
-      </c>
-      <c r="C11">
-        <v>139</v>
-      </c>
-      <c r="D11">
+      <c r="E24">
+        <v>99.3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25">
+        <v>125</v>
+      </c>
+      <c r="C25">
+        <v>124</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25">
+        <v>99.2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" t="s">
+        <v>5</v>
+      </c>
+      <c r="B26">
+        <v>683</v>
+      </c>
+      <c r="C26">
+        <v>675</v>
+      </c>
+      <c r="D26">
+        <v>8</v>
+      </c>
+      <c r="E26">
+        <v>98.8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27">
+        <v>177</v>
+      </c>
+      <c r="C27">
+        <v>174</v>
+      </c>
+      <c r="D27">
+        <v>3</v>
+      </c>
+      <c r="E27">
+        <v>98.3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B28">
+        <v>57</v>
+      </c>
+      <c r="C28">
+        <v>56</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>98.2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29">
+        <v>44</v>
+      </c>
+      <c r="C29">
+        <v>43</v>
+      </c>
+      <c r="D29">
+        <v>1</v>
+      </c>
+      <c r="E29">
+        <v>97.7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" t="s">
+        <v>24</v>
+      </c>
+      <c r="B30">
+        <v>70</v>
+      </c>
+      <c r="C30">
+        <v>68</v>
+      </c>
+      <c r="D30">
         <v>2</v>
       </c>
-      <c r="E11">
-        <v>98.59999999999999</v>
+      <c r="E30">
+        <v>97.09999999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31">
+        <v>813</v>
+      </c>
+      <c r="C31">
+        <v>789</v>
+      </c>
+      <c r="D31">
+        <v>24</v>
+      </c>
+      <c r="E31">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B32">
+        <v>179</v>
+      </c>
+      <c r="C32">
+        <v>173</v>
+      </c>
+      <c r="D32">
+        <v>6</v>
+      </c>
+      <c r="E32">
+        <v>96.59999999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" t="s">
+        <v>2</v>
+      </c>
+      <c r="B33">
+        <v>975</v>
+      </c>
+      <c r="C33">
+        <v>931</v>
+      </c>
+      <c r="D33">
+        <v>44</v>
+      </c>
+      <c r="E33">
+        <v>95.5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" t="s">
+        <v>18</v>
+      </c>
+      <c r="B34">
+        <v>120</v>
+      </c>
+      <c r="C34">
+        <v>111</v>
+      </c>
+      <c r="D34">
+        <v>9</v>
+      </c>
+      <c r="E34">
+        <v>92.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" t="s">
+        <v>6</v>
+      </c>
+      <c r="B35">
+        <v>515</v>
+      </c>
+      <c r="C35">
+        <v>461</v>
+      </c>
+      <c r="D35">
+        <v>54</v>
+      </c>
+      <c r="E35">
+        <v>89.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Izvestaj (IZVESTAJ.md + IZVESTAJ.docx) + normalizacija brenda u ciscenju
Kompletan izvestaj sa svim sekcijama postavke, stvarnim brojevima i evaluacijom modela (R2/RMSE, silhouette, krive ucenja, 2 primera preporuka); Word verzija sa ugradjenim grafikonima. Normalizacija brenda (velika slova) spaja Vox/VOX itd. - cistiji top brendovi. .docbuild gitignore-ovan.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/izvestaj/upiti_rezultati.xlsx
+++ b/izvestaj/upiti_rezultati.xlsx
@@ -136,34 +136,34 @@
     <t>brend</t>
   </si>
   <si>
-    <t>Gorenje</t>
-  </si>
-  <si>
-    <t>Beko</t>
-  </si>
-  <si>
-    <t>Bosch</t>
-  </si>
-  <si>
-    <t>Vox</t>
-  </si>
-  <si>
-    <t>Candy</t>
+    <t>GORENJE</t>
   </si>
   <si>
     <t>VOX</t>
   </si>
   <si>
-    <t>Philips</t>
-  </si>
-  <si>
-    <t>Haier</t>
-  </si>
-  <si>
-    <t>Samsung</t>
-  </si>
-  <si>
-    <t>Electrolux</t>
+    <t>BOSCH</t>
+  </si>
+  <si>
+    <t>BEKO</t>
+  </si>
+  <si>
+    <t>CANDY</t>
+  </si>
+  <si>
+    <t>PHILIPS</t>
+  </si>
+  <si>
+    <t>HAIER</t>
+  </si>
+  <si>
+    <t>SAMSUNG</t>
+  </si>
+  <si>
+    <t>WHIRLPOOL</t>
+  </si>
+  <si>
+    <t>ELECTROLUX</t>
   </si>
   <si>
     <t>naziv</t>
@@ -268,7 +268,7 @@
     <t>Hisense Smart televizor 75A7Q</t>
   </si>
   <si>
-    <t>Hisense</t>
+    <t>HISENSE</t>
   </si>
   <si>
     <t>LG</t>
@@ -307,25 +307,25 @@
     <t>procenat_klasa_a</t>
   </si>
   <si>
-    <t>Alfa Plam</t>
-  </si>
-  <si>
-    <t>Milan Blagojevic</t>
-  </si>
-  <si>
-    <t>Roborock</t>
-  </si>
-  <si>
-    <t>Aeg</t>
-  </si>
-  <si>
-    <t>Dyson</t>
+    <t>ALFA PLAM</t>
+  </si>
+  <si>
+    <t>MILAN BLAGOJEVIC</t>
+  </si>
+  <si>
+    <t>ROBOROCK</t>
+  </si>
+  <si>
+    <t>AEG</t>
+  </si>
+  <si>
+    <t>DYSON</t>
   </si>
   <si>
     <t>TCL</t>
   </si>
   <si>
-    <t>Dreame</t>
+    <t>DREAME</t>
   </si>
   <si>
     <t>na_lageru</t>
@@ -1038,7 +1038,7 @@
         <v>37</v>
       </c>
       <c r="B2">
-        <v>833</v>
+        <v>857</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -1046,7 +1046,7 @@
         <v>38</v>
       </c>
       <c r="B3">
-        <v>536</v>
+        <v>800</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -1054,7 +1054,7 @@
         <v>39</v>
       </c>
       <c r="B4">
-        <v>527</v>
+        <v>565</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -1062,7 +1062,7 @@
         <v>40</v>
       </c>
       <c r="B5">
-        <v>439</v>
+        <v>557</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -1070,7 +1070,7 @@
         <v>41</v>
       </c>
       <c r="B6">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -1078,7 +1078,7 @@
         <v>42</v>
       </c>
       <c r="B7">
-        <v>361</v>
+        <v>284</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -1086,7 +1086,7 @@
         <v>43</v>
       </c>
       <c r="B8">
-        <v>280</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -1094,7 +1094,7 @@
         <v>44</v>
       </c>
       <c r="B9">
-        <v>192</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -1102,7 +1102,7 @@
         <v>45</v>
       </c>
       <c r="B10">
-        <v>174</v>
+        <v>169</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -1196,7 +1196,7 @@
         <v>52</v>
       </c>
       <c r="B3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C3">
         <v>119999</v>
@@ -1213,7 +1213,7 @@
         <v>53</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C4">
         <v>119844</v>
@@ -1281,7 +1281,7 @@
         <v>57</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C8">
         <v>109999</v>
@@ -1394,7 +1394,7 @@
         <v>64</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C15">
         <v>99999</v>
@@ -1411,7 +1411,7 @@
         <v>65</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C16">
         <v>99999</v>
@@ -1462,7 +1462,7 @@
         <v>68</v>
       </c>
       <c r="B19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C19">
         <v>89999</v>
@@ -1479,7 +1479,7 @@
         <v>69</v>
       </c>
       <c r="B20" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C20">
         <v>89999</v>
@@ -1496,7 +1496,7 @@
         <v>70</v>
       </c>
       <c r="B21" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C21">
         <v>89999</v>
@@ -1513,7 +1513,7 @@
         <v>71</v>
       </c>
       <c r="B22" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C22">
         <v>89999</v>
@@ -1530,7 +1530,7 @@
         <v>72</v>
       </c>
       <c r="B23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C23">
         <v>89977</v>
@@ -1564,7 +1564,7 @@
         <v>74</v>
       </c>
       <c r="B25" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C25">
         <v>84999</v>
@@ -2688,36 +2688,36 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="B5">
-        <v>29</v>
+        <v>194</v>
       </c>
       <c r="C5">
-        <v>68982</v>
+        <v>67990</v>
       </c>
       <c r="D5">
-        <v>17999</v>
+        <v>5999</v>
       </c>
       <c r="E5">
-        <v>115999</v>
+        <v>119999</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>97</v>
       </c>
       <c r="B6">
-        <v>192</v>
+        <v>30</v>
       </c>
       <c r="C6">
-        <v>68022</v>
+        <v>67479</v>
       </c>
       <c r="D6">
-        <v>5999</v>
+        <v>17999</v>
       </c>
       <c r="E6">
-        <v>119999</v>
+        <v>115999</v>
       </c>
     </row>
     <row r="7" spans="1:5">

</xml_diff>

<commit_message>
GUI fiksevi: citljiv graf kategorija (horizontalni top-18), predict uppercase brend, granice tehnickih atributa (resava klaster-singleton)
1) Pregled baze: horizontalni bar top-18 umesto 34 necitljiva stuba. 2) Regresija predict: uppercase brend da se uskladi sa normalizovanom bazom (primer 'Samsung' vise ne baca gresku). 3) cisti_podatke: granice fizicki mogucih tehnickih vrednosti (frizider 2069l -> NULL) - K=4 sad daje 4 balansirana klastera umesto singletona.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/izvestaj/upiti_rezultati.xlsx
+++ b/izvestaj/upiti_rezultati.xlsx
@@ -1009,10 +1009,10 @@
         <v>107</v>
       </c>
       <c r="B4">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C4">
-        <v>84230</v>
+        <v>86222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>